<commit_message>
Load missing Gmail expenses into CIUDAD, OHIGGINS, BONORINO, AVA and regenerate SOL master.
Includes Jul–Sep expensas, utilities (Telecentro/Metrogas/Edenor/Edesur), AVA cuotas 10–11 with MEP TC, GPS/Almacén rows, and MP No Gasto card payments.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +195,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1287,29 +1288,57 @@
           <t>agosto 2026</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+      <c r="C11" s="19" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="D11" s="31" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>4110.29</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>3134720</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>3134720</v>
+      </c>
       <c r="J11" s="20" t="n">
-        <v>49449457</v>
-      </c>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="19" t="n"/>
+        <v>55718897</v>
+      </c>
+      <c r="K11" s="19" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
       <c r="M11" s="19" t="n"/>
       <c r="N11" s="19" t="n"/>
       <c r="O11" s="19" t="n"/>
       <c r="P11" s="19" t="n"/>
-      <c r="Q11" s="19" t="n"/>
+      <c r="Q11" s="19" t="inlineStr">
+        <is>
+          <t>IPC/CAC pendiente</t>
+        </is>
+      </c>
       <c r="R11" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S11" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S11" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 25-ago + pago 7-sep · TC MEP venta api.argentinadatos bolsa</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n">
@@ -1320,15 +1349,19 @@
           <t>septiembre 2026</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
+      <c r="C12" s="19" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="D12" s="31" t="n">
+        <v>46300</v>
+      </c>
       <c r="E12" s="19" t="n"/>
       <c r="F12" s="19" t="n"/>
       <c r="G12" s="19" t="n"/>
       <c r="H12" s="19" t="n"/>
       <c r="I12" s="19" t="n"/>
       <c r="J12" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K12" s="19" t="n"/>
       <c r="L12" s="19" t="n"/>
@@ -1342,7 +1375,11 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="S12" s="19" t="n"/>
+      <c r="S12" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 24-sep aviso · aún no pagada</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n">
@@ -1361,7 +1398,7 @@
       <c r="H13" s="19" t="n"/>
       <c r="I13" s="19" t="n"/>
       <c r="J13" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K13" s="19" t="n"/>
       <c r="L13" s="19" t="n"/>
@@ -1394,7 +1431,7 @@
       <c r="H14" s="19" t="n"/>
       <c r="I14" s="19" t="n"/>
       <c r="J14" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K14" s="19" t="n"/>
       <c r="L14" s="19" t="n"/>
@@ -1427,7 +1464,7 @@
       <c r="H15" s="19" t="n"/>
       <c r="I15" s="19" t="n"/>
       <c r="J15" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K15" s="19" t="n"/>
       <c r="L15" s="19" t="n"/>
@@ -1460,7 +1497,7 @@
       <c r="H16" s="19" t="n"/>
       <c r="I16" s="19" t="n"/>
       <c r="J16" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K16" s="19" t="n"/>
       <c r="L16" s="19" t="n"/>
@@ -1493,7 +1530,7 @@
       <c r="H17" s="19" t="n"/>
       <c r="I17" s="19" t="n"/>
       <c r="J17" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K17" s="19" t="n"/>
       <c r="L17" s="19" t="n"/>
@@ -1526,7 +1563,7 @@
       <c r="H18" s="19" t="n"/>
       <c r="I18" s="19" t="n"/>
       <c r="J18" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K18" s="19" t="n"/>
       <c r="L18" s="19" t="n"/>
@@ -1559,7 +1596,7 @@
       <c r="H19" s="19" t="n"/>
       <c r="I19" s="19" t="n"/>
       <c r="J19" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K19" s="19" t="n"/>
       <c r="L19" s="19" t="n"/>
@@ -1592,7 +1629,7 @@
       <c r="H20" s="19" t="n"/>
       <c r="I20" s="19" t="n"/>
       <c r="J20" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K20" s="19" t="n"/>
       <c r="L20" s="19" t="n"/>
@@ -1625,7 +1662,7 @@
       <c r="H21" s="19" t="n"/>
       <c r="I21" s="19" t="n"/>
       <c r="J21" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K21" s="19" t="n"/>
       <c r="L21" s="19" t="n"/>
@@ -1658,7 +1695,7 @@
       <c r="H22" s="19" t="n"/>
       <c r="I22" s="19" t="n"/>
       <c r="J22" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K22" s="19" t="n"/>
       <c r="L22" s="19" t="n"/>
@@ -1691,7 +1728,7 @@
       <c r="H23" s="19" t="n"/>
       <c r="I23" s="19" t="n"/>
       <c r="J23" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K23" s="19" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -1724,7 +1761,7 @@
       <c r="H24" s="19" t="n"/>
       <c r="I24" s="19" t="n"/>
       <c r="J24" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K24" s="19" t="n"/>
       <c r="L24" s="19" t="n"/>
@@ -1757,7 +1794,7 @@
       <c r="H25" s="19" t="n"/>
       <c r="I25" s="19" t="n"/>
       <c r="J25" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K25" s="19" t="n"/>
       <c r="L25" s="19" t="n"/>
@@ -1790,7 +1827,7 @@
       <c r="H26" s="19" t="n"/>
       <c r="I26" s="19" t="n"/>
       <c r="J26" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K26" s="19" t="n"/>
       <c r="L26" s="19" t="n"/>
@@ -1823,7 +1860,7 @@
       <c r="H27" s="19" t="n"/>
       <c r="I27" s="19" t="n"/>
       <c r="J27" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K27" s="19" t="n"/>
       <c r="L27" s="19" t="n"/>
@@ -1856,7 +1893,7 @@
       <c r="H28" s="19" t="n"/>
       <c r="I28" s="19" t="n"/>
       <c r="J28" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K28" s="19" t="n"/>
       <c r="L28" s="19" t="n"/>
@@ -1889,7 +1926,7 @@
       <c r="H29" s="19" t="n"/>
       <c r="I29" s="19" t="n"/>
       <c r="J29" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K29" s="19" t="n"/>
       <c r="L29" s="19" t="n"/>
@@ -1922,7 +1959,7 @@
       <c r="H30" s="19" t="n"/>
       <c r="I30" s="19" t="n"/>
       <c r="J30" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K30" s="19" t="n"/>
       <c r="L30" s="19" t="n"/>
@@ -1955,7 +1992,7 @@
       <c r="H31" s="19" t="n"/>
       <c r="I31" s="19" t="n"/>
       <c r="J31" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K31" s="19" t="n"/>
       <c r="L31" s="19" t="n"/>
@@ -1988,7 +2025,7 @@
       <c r="H32" s="19" t="n"/>
       <c r="I32" s="19" t="n"/>
       <c r="J32" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K32" s="19" t="n"/>
       <c r="L32" s="19" t="n"/>
@@ -2021,7 +2058,7 @@
       <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
       <c r="J33" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
@@ -2037,6 +2074,7 @@
       </c>
       <c r="S33" s="19" t="n"/>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="25" t="inlineStr">
         <is>
@@ -2056,6 +2094,7 @@
         <v>24724726</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="25" t="inlineStr">
         <is>
@@ -2140,7 +2179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2482,6 +2521,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>agosto 2026</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>IPC/CAC pendiente</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>IPC/CAC julio 2026 pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2647,7 +2710,9 @@
       <c r="J5" s="5" t="n">
         <v>6005392</v>
       </c>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>6269440</v>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
@@ -3381,16 +3446,44 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="9" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Cuota 10 · agosto 2026</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3134720 en Gasto Personal Sol (CIUDAD) · TC MEP venta 1525.3 (2026-09-04)</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>

</xml_diff>

<commit_message>
Load September 2026 expenses from Gmail sources.
Pull expensas, utilities, AVA cuota 10, and partial Almacén/GPS items
from official Gmail PDFs and BBVA/MP alerts; document remaining gaps
(MP settlement, BBVA statement PDFs, TC MP resumen).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +195,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1284,18 +1285,32 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>agosto 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+          <t>septiembre 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="D11" s="31" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>1525.39</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>4110.06</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>3134720</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>3134720</v>
+      </c>
       <c r="J11" s="20" t="n">
-        <v>49449457</v>
+        <v>55718897</v>
       </c>
       <c r="K11" s="19" t="n"/>
       <c r="L11" s="19" t="n"/>
@@ -2648,7 +2663,9 @@
         <v>6005392</v>
       </c>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
+      <c r="L5" s="5" t="n">
+        <v>6269440</v>
+      </c>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
@@ -3381,16 +3398,44 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="9" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Cuota 10 · septiembre 2026</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3134720 en Gasto Personal Sol (CIUDAD) · TC MEP venta 1525.39</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>

</xml_diff>

<commit_message>
Cargar AVA cuota 11 octubre (factura Cobranza, PENDIENTE)
Monto $6.550.413 · vto 05/10/2026 · TC MEP 1549.26 (02/10) ·
50% Sol $3.275.207 en cashflow PENDIENTE (aún no GPS). Sincroniza
cuota 10 PAGADO en Cashflow Compromisos.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +196,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1312,8 +1313,14 @@
       <c r="J11" s="20" t="n">
         <v>55718897</v>
       </c>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="19" t="n"/>
+      <c r="K11" s="19" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
       <c r="M11" s="19" t="n"/>
       <c r="N11" s="19" t="n"/>
       <c r="O11" s="19" t="n"/>
@@ -1321,10 +1328,14 @@
       <c r="Q11" s="19" t="n"/>
       <c r="R11" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S11" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S11" s="19" t="inlineStr">
+        <is>
+          <t>Gmail factura/recibo 07/09/2026 · TC MEP Rava cierre 1525.39</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n">
@@ -1332,32 +1343,60 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>septiembre 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
+          <t>octubre 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="D12" s="31" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1549.26</v>
+      </c>
+      <c r="F12" s="31" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>4228.09</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>3275207</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>3275206</v>
+      </c>
       <c r="J12" s="20" t="n">
-        <v>49449457</v>
-      </c>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
+        <v>62269310</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="L12" s="19" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
       <c r="M12" s="19" t="n"/>
       <c r="N12" s="19" t="n"/>
       <c r="O12" s="19" t="n"/>
       <c r="P12" s="19" t="n"/>
-      <c r="Q12" s="19" t="n"/>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>IPC/CAC sept pendiente</t>
+        </is>
+      </c>
       <c r="R12" s="19" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="S12" s="19" t="n"/>
+      <c r="S12" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Cobranza 24/09/2026 · TC MEP Rava cierre 02/10 1549.26 (pre-vto 05/10)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n">
@@ -1376,7 +1415,7 @@
       <c r="H13" s="19" t="n"/>
       <c r="I13" s="19" t="n"/>
       <c r="J13" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K13" s="19" t="n"/>
       <c r="L13" s="19" t="n"/>
@@ -1409,7 +1448,7 @@
       <c r="H14" s="19" t="n"/>
       <c r="I14" s="19" t="n"/>
       <c r="J14" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K14" s="19" t="n"/>
       <c r="L14" s="19" t="n"/>
@@ -1442,7 +1481,7 @@
       <c r="H15" s="19" t="n"/>
       <c r="I15" s="19" t="n"/>
       <c r="J15" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K15" s="19" t="n"/>
       <c r="L15" s="19" t="n"/>
@@ -1475,7 +1514,7 @@
       <c r="H16" s="19" t="n"/>
       <c r="I16" s="19" t="n"/>
       <c r="J16" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K16" s="19" t="n"/>
       <c r="L16" s="19" t="n"/>
@@ -1508,7 +1547,7 @@
       <c r="H17" s="19" t="n"/>
       <c r="I17" s="19" t="n"/>
       <c r="J17" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K17" s="19" t="n"/>
       <c r="L17" s="19" t="n"/>
@@ -1541,7 +1580,7 @@
       <c r="H18" s="19" t="n"/>
       <c r="I18" s="19" t="n"/>
       <c r="J18" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K18" s="19" t="n"/>
       <c r="L18" s="19" t="n"/>
@@ -1574,7 +1613,7 @@
       <c r="H19" s="19" t="n"/>
       <c r="I19" s="19" t="n"/>
       <c r="J19" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K19" s="19" t="n"/>
       <c r="L19" s="19" t="n"/>
@@ -1607,7 +1646,7 @@
       <c r="H20" s="19" t="n"/>
       <c r="I20" s="19" t="n"/>
       <c r="J20" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K20" s="19" t="n"/>
       <c r="L20" s="19" t="n"/>
@@ -1640,7 +1679,7 @@
       <c r="H21" s="19" t="n"/>
       <c r="I21" s="19" t="n"/>
       <c r="J21" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K21" s="19" t="n"/>
       <c r="L21" s="19" t="n"/>
@@ -1673,7 +1712,7 @@
       <c r="H22" s="19" t="n"/>
       <c r="I22" s="19" t="n"/>
       <c r="J22" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K22" s="19" t="n"/>
       <c r="L22" s="19" t="n"/>
@@ -1706,7 +1745,7 @@
       <c r="H23" s="19" t="n"/>
       <c r="I23" s="19" t="n"/>
       <c r="J23" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K23" s="19" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -1739,7 +1778,7 @@
       <c r="H24" s="19" t="n"/>
       <c r="I24" s="19" t="n"/>
       <c r="J24" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K24" s="19" t="n"/>
       <c r="L24" s="19" t="n"/>
@@ -1772,7 +1811,7 @@
       <c r="H25" s="19" t="n"/>
       <c r="I25" s="19" t="n"/>
       <c r="J25" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K25" s="19" t="n"/>
       <c r="L25" s="19" t="n"/>
@@ -1805,7 +1844,7 @@
       <c r="H26" s="19" t="n"/>
       <c r="I26" s="19" t="n"/>
       <c r="J26" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K26" s="19" t="n"/>
       <c r="L26" s="19" t="n"/>
@@ -1838,7 +1877,7 @@
       <c r="H27" s="19" t="n"/>
       <c r="I27" s="19" t="n"/>
       <c r="J27" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K27" s="19" t="n"/>
       <c r="L27" s="19" t="n"/>
@@ -1871,7 +1910,7 @@
       <c r="H28" s="19" t="n"/>
       <c r="I28" s="19" t="n"/>
       <c r="J28" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K28" s="19" t="n"/>
       <c r="L28" s="19" t="n"/>
@@ -1904,7 +1943,7 @@
       <c r="H29" s="19" t="n"/>
       <c r="I29" s="19" t="n"/>
       <c r="J29" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K29" s="19" t="n"/>
       <c r="L29" s="19" t="n"/>
@@ -1937,7 +1976,7 @@
       <c r="H30" s="19" t="n"/>
       <c r="I30" s="19" t="n"/>
       <c r="J30" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K30" s="19" t="n"/>
       <c r="L30" s="19" t="n"/>
@@ -1970,7 +2009,7 @@
       <c r="H31" s="19" t="n"/>
       <c r="I31" s="19" t="n"/>
       <c r="J31" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K31" s="19" t="n"/>
       <c r="L31" s="19" t="n"/>
@@ -2003,7 +2042,7 @@
       <c r="H32" s="19" t="n"/>
       <c r="I32" s="19" t="n"/>
       <c r="J32" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K32" s="19" t="n"/>
       <c r="L32" s="19" t="n"/>
@@ -2036,7 +2075,7 @@
       <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
       <c r="J33" s="20" t="n">
-        <v>49449457</v>
+        <v>62269310</v>
       </c>
       <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
@@ -2052,6 +2091,7 @@
       </c>
       <c r="S33" s="19" t="n"/>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="25" t="inlineStr">
         <is>
@@ -2071,6 +2111,7 @@
         <v>24724726</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="25" t="inlineStr">
         <is>
@@ -2155,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2494,6 +2535,52 @@
       <c r="I9" t="inlineStr">
         <is>
           <t>IPC ref=1.9%; falta CAC del mes 2026-06 para cerrar IPC+CAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>septiembre 2026</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>IPC/CAC ago pendiente</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Falta IPC+CAC mes ref 2026-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>octubre 2026</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>IPC/CAC sept pendiente</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Cuota +4.48% vs cuota 10; falta IPC+CAC mes ref 2026-09</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2753,9 @@
       <c r="L5" s="5" t="n">
         <v>6269440</v>
       </c>
-      <c r="M5" s="5" t="n"/>
+      <c r="M5" s="5" t="n">
+        <v>6550413</v>
+      </c>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5">
@@ -3043,7 +3132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4541,6 +4630,44 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="32" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cuota 11 · octubre 2026 · PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Pendiente / TC MEP</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Total cuota factura Cobranza 24/09. 50% Sol=$3,275,207 (aún NO en GPS hasta pagar) · TC MEP venta 1549.26 (02/10)</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Load AVA cuota 12 octubre 2026 ($6,550,413) paid via Mercado Pago.
Record the Oct 5 transfer to Fideicomiso Ava Palpa, value at MEP venta 1551.9, mirror 50% Sol into GPS/Cashflow/SOL. Septiembre (cuota 11) remains pending without invoice.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -1388,29 +1388,55 @@
           <t>octubre 2026</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
+      <c r="C13" s="19" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="D13" s="31" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>1551.9</v>
+      </c>
+      <c r="F13" s="31" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>4220.9</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>3275207</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>3275206</v>
+      </c>
       <c r="J13" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K13" s="19" t="n"/>
-      <c r="L13" s="19" t="n"/>
+      <c r="L13" s="19" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
       <c r="M13" s="19" t="n"/>
       <c r="N13" s="19" t="n"/>
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
-      <c r="Q13" s="19" t="n"/>
+      <c r="Q13" s="19" t="inlineStr">
+        <is>
+          <t>IPC/CAC sept pendiente; Δ vs cuota 11 N/D (sin factura)</t>
+        </is>
+      </c>
       <c r="R13" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S13" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S13" s="19" t="inlineStr">
+        <is>
+          <t>MEP bolsa venta (argentinadatos) 2026-10-05 = 1551.9 · abonada 2026-10-05 MP op 181443753207 · transferencia Maria Soledad Sanes → Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n">
@@ -1429,7 +1455,7 @@
       <c r="H14" s="19" t="n"/>
       <c r="I14" s="19" t="n"/>
       <c r="J14" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K14" s="19" t="n"/>
       <c r="L14" s="19" t="n"/>
@@ -1462,7 +1488,7 @@
       <c r="H15" s="19" t="n"/>
       <c r="I15" s="19" t="n"/>
       <c r="J15" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K15" s="19" t="n"/>
       <c r="L15" s="19" t="n"/>
@@ -1495,7 +1521,7 @@
       <c r="H16" s="19" t="n"/>
       <c r="I16" s="19" t="n"/>
       <c r="J16" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K16" s="19" t="n"/>
       <c r="L16" s="19" t="n"/>
@@ -1528,7 +1554,7 @@
       <c r="H17" s="19" t="n"/>
       <c r="I17" s="19" t="n"/>
       <c r="J17" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K17" s="19" t="n"/>
       <c r="L17" s="19" t="n"/>
@@ -1561,7 +1587,7 @@
       <c r="H18" s="19" t="n"/>
       <c r="I18" s="19" t="n"/>
       <c r="J18" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K18" s="19" t="n"/>
       <c r="L18" s="19" t="n"/>
@@ -1594,7 +1620,7 @@
       <c r="H19" s="19" t="n"/>
       <c r="I19" s="19" t="n"/>
       <c r="J19" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K19" s="19" t="n"/>
       <c r="L19" s="19" t="n"/>
@@ -1627,7 +1653,7 @@
       <c r="H20" s="19" t="n"/>
       <c r="I20" s="19" t="n"/>
       <c r="J20" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K20" s="19" t="n"/>
       <c r="L20" s="19" t="n"/>
@@ -1660,7 +1686,7 @@
       <c r="H21" s="19" t="n"/>
       <c r="I21" s="19" t="n"/>
       <c r="J21" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K21" s="19" t="n"/>
       <c r="L21" s="19" t="n"/>
@@ -1693,7 +1719,7 @@
       <c r="H22" s="19" t="n"/>
       <c r="I22" s="19" t="n"/>
       <c r="J22" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K22" s="19" t="n"/>
       <c r="L22" s="19" t="n"/>
@@ -1726,7 +1752,7 @@
       <c r="H23" s="19" t="n"/>
       <c r="I23" s="19" t="n"/>
       <c r="J23" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K23" s="19" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -1759,7 +1785,7 @@
       <c r="H24" s="19" t="n"/>
       <c r="I24" s="19" t="n"/>
       <c r="J24" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K24" s="19" t="n"/>
       <c r="L24" s="19" t="n"/>
@@ -1792,7 +1818,7 @@
       <c r="H25" s="19" t="n"/>
       <c r="I25" s="19" t="n"/>
       <c r="J25" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K25" s="19" t="n"/>
       <c r="L25" s="19" t="n"/>
@@ -1825,7 +1851,7 @@
       <c r="H26" s="19" t="n"/>
       <c r="I26" s="19" t="n"/>
       <c r="J26" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K26" s="19" t="n"/>
       <c r="L26" s="19" t="n"/>
@@ -1858,7 +1884,7 @@
       <c r="H27" s="19" t="n"/>
       <c r="I27" s="19" t="n"/>
       <c r="J27" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K27" s="19" t="n"/>
       <c r="L27" s="19" t="n"/>
@@ -1891,7 +1917,7 @@
       <c r="H28" s="19" t="n"/>
       <c r="I28" s="19" t="n"/>
       <c r="J28" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K28" s="19" t="n"/>
       <c r="L28" s="19" t="n"/>
@@ -1924,7 +1950,7 @@
       <c r="H29" s="19" t="n"/>
       <c r="I29" s="19" t="n"/>
       <c r="J29" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K29" s="19" t="n"/>
       <c r="L29" s="19" t="n"/>
@@ -1957,7 +1983,7 @@
       <c r="H30" s="19" t="n"/>
       <c r="I30" s="19" t="n"/>
       <c r="J30" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K30" s="19" t="n"/>
       <c r="L30" s="19" t="n"/>
@@ -1990,7 +2016,7 @@
       <c r="H31" s="19" t="n"/>
       <c r="I31" s="19" t="n"/>
       <c r="J31" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K31" s="19" t="n"/>
       <c r="L31" s="19" t="n"/>
@@ -2023,7 +2049,7 @@
       <c r="H32" s="19" t="n"/>
       <c r="I32" s="19" t="n"/>
       <c r="J32" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K32" s="19" t="n"/>
       <c r="L32" s="19" t="n"/>
@@ -2056,7 +2082,7 @@
       <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
       <c r="J33" s="20" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
@@ -2079,16 +2105,16 @@
         </is>
       </c>
       <c r="C35" s="26" t="n">
-        <v>55627979</v>
+        <v>62178392</v>
       </c>
       <c r="G35" s="27" t="n">
-        <v>37698.92</v>
+        <v>41919.82</v>
       </c>
       <c r="H35" s="14" t="n">
-        <v>27813992</v>
+        <v>31089199</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>27813987</v>
+        <v>31089193</v>
       </c>
     </row>
     <row r="37">
@@ -2175,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2546,6 +2572,26 @@
       <c r="I10" t="inlineStr">
         <is>
           <t>Falta IPC y CAC del mes 2026-07 para cerrar IPC+CAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>octubre 2026</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>IPC/CAC sept pendiente</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pagada $6,550,413. Cuota 11 (sep) sin factura — %Δ mes a mes N/D. Vs última pagada (ago): +6.02%</t>
         </is>
       </c>
     </row>
@@ -2595,6 +2641,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2718,7 +2765,9 @@
         <v>6178522</v>
       </c>
       <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
+      <c r="M5" s="5" t="n">
+        <v>6550413</v>
+      </c>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5">
@@ -3490,16 +3539,44 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="4" t="n"/>
+      <c r="A12" s="9" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Cuota 12 · octubre 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3,275,207 en Gasto Personal Sol (CIUDAD). Abonada 2026-10-05. MP op 181443753207. TC MEP venta 1551.9 (2026-10-05). ID 1LMP68NKKM3D5DKKNR7OEV</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>

</xml_diff>

<commit_message>
Expose AVA MEP seller FX as payment-day rate in Excel.
Clarify Cuotas/Detalle columns for TC MEP venta on the cuota payment date (octubre 2026 = 1551.9 on 2026-10-05).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +196,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,14 +610,14 @@
           <t>Fecha vencimiento</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
-        <is>
-          <t>TC MEP venta</t>
-        </is>
-      </c>
-      <c r="F1" s="18" t="inlineStr">
-        <is>
-          <t>Fecha cotización MEP</t>
+      <c r="E1" s="32" t="inlineStr">
+        <is>
+          <t>TC MEP venta (día pago)</t>
+        </is>
+      </c>
+      <c r="F1" s="32" t="inlineStr">
+        <is>
+          <t>Fecha día pago (cotiz. MEP)</t>
         </is>
       </c>
       <c r="G1" s="18" t="inlineStr">
@@ -1434,7 +1438,7 @@
       </c>
       <c r="S13" s="19" t="inlineStr">
         <is>
-          <t>MEP bolsa venta (argentinadatos) 2026-10-05 = 1551.9 · abonada 2026-10-05 MP op 181443753207 · transferencia Maria Soledad Sanes → Fideicomiso Ava Palpa</t>
+          <t>TC MEP VENDEDOR (venta) día de pago 2026-10-05 = 1551.9 (argentinadatos dólar bolsa) · abonada 2026-10-05 MP op 181443753207 · transferencia Maria Soledad Sanes → Fideicomiso Ava Palpa</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2131,7 @@
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>TC MEP: siempre dólar bolsa (MEP) tipo VENDEDOR (venta) de api.argentinadatos.com en la fecha de vencimiento de la cuota (si no hay rueda, día hábil anterior).</t>
+          <t>TC MEP: siempre dólar bolsa (MEP) tipo VENDEDOR (venta) del DÍA DE PAGO de la cuota (api.argentinadatos.com). Si no hay rueda ese día, último hábil anterior. Valor USD = Monto ARS ÷ TC MEP venta.</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2645,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3144,7 +3147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3217,6 +3220,16 @@
           <t>Mes</t>
         </is>
       </c>
+      <c r="K3" s="25" t="inlineStr">
+        <is>
+          <t>TC MEP venta (día pago)</t>
+        </is>
+      </c>
+      <c r="L3" s="25" t="inlineStr">
+        <is>
+          <t>Fecha día pago</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="n">
@@ -3257,6 +3270,12 @@
           <t>Enero</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>1501.8</v>
+      </c>
+      <c r="L4" s="33" t="n">
+        <v>46027</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="n">
@@ -3297,6 +3316,12 @@
           <t>Febrero</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>1459.7</v>
+      </c>
+      <c r="L5" s="33" t="n">
+        <v>46057</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="n">
@@ -3337,6 +3362,12 @@
           <t>Marzo</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>1429.9</v>
+      </c>
+      <c r="L6" s="33" t="n">
+        <v>46085</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="n">
@@ -3377,6 +3408,12 @@
           <t>Abril</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>1430.6</v>
+      </c>
+      <c r="L7" s="33" t="n">
+        <v>46118</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="n">
@@ -3417,6 +3454,12 @@
           <t>Mayo</t>
         </is>
       </c>
+      <c r="K8" t="n">
+        <v>1448.5</v>
+      </c>
+      <c r="L8" s="33" t="n">
+        <v>46148</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="n">
@@ -3457,6 +3500,12 @@
           <t>Junio</t>
         </is>
       </c>
+      <c r="K9" t="n">
+        <v>1461.4</v>
+      </c>
+      <c r="L9" s="33" t="n">
+        <v>46178</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="n">
@@ -3497,6 +3546,12 @@
           <t>Julio</t>
         </is>
       </c>
+      <c r="K10" t="n">
+        <v>1525.1</v>
+      </c>
+      <c r="L10" s="33" t="n">
+        <v>46209</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -3537,6 +3592,12 @@
           <t>Agosto</t>
         </is>
       </c>
+      <c r="K11" t="n">
+        <v>1524.5</v>
+      </c>
+      <c r="L11" s="33" t="n">
+        <v>46238</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -3576,6 +3637,12 @@
         <is>
           <t>Octubre</t>
         </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1551.9</v>
+      </c>
+      <c r="L12" s="33" t="n">
+        <v>46300</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Fill monthly utilities gaps from Gmail across CIUDAD, OHIGGINS, BONORINO, AVA.
Fixes Telecentro Aug BBVA amount, loads Edenor/Spotify/Personal/Edesur/expensas Sep, and AVA cuota 11; clears Telecentro placeholder months without cobro.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +196,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2074,7 +2075,6 @@
       </c>
       <c r="S33" s="19" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="B35" s="25" t="inlineStr">
         <is>
@@ -2094,7 +2094,6 @@
         <v>24724726</v>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="B37" s="25" t="inlineStr">
         <is>
@@ -2179,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2544,7 +2543,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2713,7 +2711,9 @@
       <c r="K5" s="5" t="n">
         <v>6269440</v>
       </c>
-      <c r="L5" s="5" t="n"/>
+      <c r="L5" s="5" t="n">
+        <v>6550413</v>
+      </c>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
@@ -3091,7 +3091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3113,6 +3113,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -4589,6 +4590,44 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="32" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cuota 11 · septiembre 2026</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>PENDIENTE · aviso Gmail Sancor</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol TBD al pagar · venc. 05/10/2026</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Verificar mails BBVA/AVA y actualizar planillas; Chris no pagó septiembre.
Marca cuotas BBVA jun–sep 2026 como PAGADO, carga utilidades y AVA 10–13,
registra liquidación septiembre sin pago de Chris, y regenera el maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -21,11 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -560,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S45"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1287,13 +1286,27 @@
           <t>agosto 2026</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+      <c r="C11" s="19" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>1518.45</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>46239</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>4068.97</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>3089261</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>3089261</v>
+      </c>
       <c r="J11" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1306,10 +1319,14 @@
       <c r="Q11" s="19" t="n"/>
       <c r="R11" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S11" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S11" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 22/07 · MEP Rava 1518.45</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n">
@@ -1320,13 +1337,27 @@
           <t>septiembre 2026</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
+      <c r="C12" s="19" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1525.39</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>4110.06</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>3134720</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>3134720</v>
+      </c>
       <c r="J12" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1339,10 +1370,14 @@
       <c r="Q12" s="19" t="n"/>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S12" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S12" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 25/08 · MEP Rava 1525.39 · GPS OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n">
@@ -1353,13 +1388,27 @@
           <t>octubre 2026</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
+      <c r="C13" s="19" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>1538.39</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>4257.97</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>3275206</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>3275207</v>
+      </c>
       <c r="J13" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1372,10 +1421,14 @@
       <c r="Q13" s="19" t="n"/>
       <c r="R13" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S13" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S13" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 24/09 · MEP Rava 1538.39</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n">
@@ -1386,13 +1439,21 @@
           <t>noviembre 2026</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
+      <c r="C14" s="19" t="n">
+        <v>6739503</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>46330</v>
+      </c>
       <c r="E14" s="19" t="n"/>
       <c r="F14" s="19" t="n"/>
       <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
+      <c r="H14" s="19" t="n">
+        <v>3369751</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>3369752</v>
+      </c>
       <c r="J14" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1408,7 +1469,11 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="S14" s="19" t="n"/>
+      <c r="S14" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 23/10 · TC MEP TBD al vencimiento 04/11</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n">
@@ -2037,6 +2102,7 @@
       </c>
       <c r="S33" s="19" t="n"/>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="25" t="inlineStr">
         <is>
@@ -2056,6 +2122,7 @@
         <v>24724726</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="25" t="inlineStr">
         <is>
@@ -2647,10 +2714,18 @@
       <c r="J5" s="5" t="n">
         <v>6005392</v>
       </c>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>6739503</v>
+      </c>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5">
         <f>SUM(D5:O5)</f>
@@ -3026,7 +3101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4496,6 +4571,138 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="16" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cuota 10 · agosto 2026</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3089261 en Gasto Personal Sol (CIUDAD). Gmail Sancor 22/07 · vto 05/08 · MEP Rava cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Cuota 11 · septiembre 2026</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3134720 en Gasto Personal Sol (CIUDAD). Gmail Sancor 25/08 · vto 04/09 · MEP Rava · ya en GPS (renum cuota 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Cuota 12 · octubre 2026</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3275206 en Gasto Personal Sol (CIUDAD). Gmail Sancor 24/09 · vto 05/10 · MEP Rava cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Cuota 13 · noviembre 2026</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>6739503</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>PENDIENTE factura</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3369751 en Gasto Personal Sol (CIUDAD). Gmail Sancor 23/10 · vto 04/11 · TC MEP pendiente hasta rueda del vencimiento</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Obligar sync a Drive 03_Finanzas_y_Gastos en toda tarea de gastos.
De ahora en más ninguna planilla queda completa solo en git: overwrite
en la raíz canónica y verificación en carpeta antes de cerrar.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AVA/Gastos_AVA_2026.xlsx
+++ b/AVA/Gastos_AVA_2026.xlsx
@@ -21,11 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -560,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S45"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1287,13 +1286,27 @@
           <t>agosto 2026</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+      <c r="C11" s="19" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>1518.45</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>46239</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>4068.97</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>3089261</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>3089261</v>
+      </c>
       <c r="J11" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1306,10 +1319,14 @@
       <c r="Q11" s="19" t="n"/>
       <c r="R11" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S11" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S11" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 22/07 · MEP Rava 1518.45</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n">
@@ -1320,13 +1337,27 @@
           <t>septiembre 2026</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
+      <c r="C12" s="19" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1525.39</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>4110.06</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>3134720</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>3134720</v>
+      </c>
       <c r="J12" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1339,10 +1370,14 @@
       <c r="Q12" s="19" t="n"/>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S12" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S12" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 25/08 · MEP Rava 1525.39 · GPS OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n">
@@ -1353,13 +1388,27 @@
           <t>octubre 2026</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
+      <c r="C13" s="19" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>1538.39</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>4257.97</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>3275206</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>3275207</v>
+      </c>
       <c r="J13" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1372,10 +1421,14 @@
       <c r="Q13" s="19" t="n"/>
       <c r="R13" s="19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="S13" s="19" t="n"/>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="S13" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 24/09 · MEP Rava 1538.39</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n">
@@ -1386,13 +1439,21 @@
           <t>noviembre 2026</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
+      <c r="C14" s="19" t="n">
+        <v>6739503</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>46330</v>
+      </c>
       <c r="E14" s="19" t="n"/>
       <c r="F14" s="19" t="n"/>
       <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
+      <c r="H14" s="19" t="n">
+        <v>3369751</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>3369752</v>
+      </c>
       <c r="J14" s="20" t="n">
         <v>49449457</v>
       </c>
@@ -1408,7 +1469,11 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="S14" s="19" t="n"/>
+      <c r="S14" s="19" t="inlineStr">
+        <is>
+          <t>Gmail Sancor 23/10 · TC MEP TBD al vencimiento 04/11</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n">
@@ -2037,6 +2102,7 @@
       </c>
       <c r="S33" s="19" t="n"/>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="25" t="inlineStr">
         <is>
@@ -2056,6 +2122,7 @@
         <v>24724726</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="25" t="inlineStr">
         <is>
@@ -2647,10 +2714,18 @@
       <c r="J5" s="5" t="n">
         <v>6005392</v>
       </c>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>6739503</v>
+      </c>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5">
         <f>SUM(D5:O5)</f>
@@ -3026,7 +3101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4496,6 +4571,138 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="16" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cuota 10 · agosto 2026</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>6178522</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3089261 en Gasto Personal Sol (CIUDAD). Gmail Sancor 22/07 · vto 05/08 · MEP Rava cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Cuota 11 · septiembre 2026</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3134720 en Gasto Personal Sol (CIUDAD). Gmail Sancor 25/08 · vto 04/09 · MEP Rava · ya en GPS (renum cuota 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Cuota 12 · octubre 2026</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>6550413</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Mercado Pago / TC MEP</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3275206 en Gasto Personal Sol (CIUDAD). Gmail Sancor 24/09 · vto 05/10 · MEP Rava cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Cuota 13 · noviembre 2026</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>6739503</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>PENDIENTE factura</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Total cuota. 50% Sol=$3369751 en Gasto Personal Sol (CIUDAD). Gmail Sancor 23/10 · vto 04/11 · TC MEP pendiente hasta rueda del vencimiento</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>